<commit_message>
Release v2.15.1: update SMS ODK forms
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/sms/example_odk_showcase_sms_send.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/sms/example_odk_showcase_sms_send.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R4740389950464a43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rcb20e52abbab48f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rf63283be72ac4efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rfadb0c8f0de84a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R694915778c944584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rc602f5cd20a1415a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -336,15 +336,15 @@
       <x:c r="D2" s="8" t="str">
         <x:v>Send a templated SMS message to a phone number</x:v>
       </x:c>
-      <x:c r="E2" s="8" t="str"/>
-      <x:c r="F2" s="8" t="str"/>
-      <x:c r="G2" s="8" t="str"/>
-      <x:c r="H2" s="8" t="str"/>
-      <x:c r="I2" s="8" t="str"/>
-      <x:c r="J2" s="8" t="str"/>
-      <x:c r="K2" s="8" t="str"/>
-      <x:c r="L2" s="8" t="str"/>
-      <x:c r="M2" s="8" t="str"/>
+      <x:c r="E2" s="8"/>
+      <x:c r="F2" s="8"/>
+      <x:c r="G2" s="8"/>
+      <x:c r="H2" s="8"/>
+      <x:c r="I2" s="8"/>
+      <x:c r="J2" s="8"/>
+      <x:c r="K2" s="8"/>
+      <x:c r="L2" s="8"/>
+      <x:c r="M2" s="8"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -362,13 +362,13 @@
       <x:c r="E3" s="8" t="str">
         <x:v>field-list</x:v>
       </x:c>
-      <x:c r="F3" s="8" t="str"/>
-      <x:c r="G3" s="8" t="str"/>
-      <x:c r="H3" s="8" t="str"/>
-      <x:c r="I3" s="8" t="str"/>
-      <x:c r="J3" s="8" t="str"/>
-      <x:c r="K3" s="8" t="str"/>
-      <x:c r="L3" s="8" t="str"/>
+      <x:c r="F3" s="8"/>
+      <x:c r="G3" s="8"/>
+      <x:c r="H3" s="8"/>
+      <x:c r="I3" s="8"/>
+      <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
+      <x:c r="L3" s="8"/>
       <x:c r="M3" s="8" t="str">
         <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='sms.send',input_sms_phone=${phone_number},input_sms_message=${sms_message_calc},return_mode='flat',input_payload_mode='FULL')</x:v>
       </x:c>
@@ -381,18 +381,20 @@
         <x:v>phone_number</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
-        <x:v>Phone number</x:v>
-      </x:c>
-      <x:c r="D4" s="8" t="str"/>
-      <x:c r="E4" s="8" t="str"/>
-      <x:c r="F4" s="8" t="str"/>
-      <x:c r="G4" s="8" t="str"/>
-      <x:c r="H4" s="8" t="str"/>
-      <x:c r="I4" s="8" t="str"/>
-      <x:c r="J4" s="8" t="str"/>
-      <x:c r="K4" s="8" t="str"/>
-      <x:c r="L4" s="8" t="str"/>
-      <x:c r="M4" s="8" t="str"/>
+        <x:v>Phone numbers (comma, semicolon, or newline separated)</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Each number receives an individual identical SMS. Duplicate numbers are sent only once.</x:v>
+      </x:c>
+      <x:c r="E4" s="8"/>
+      <x:c r="F4" s="8"/>
+      <x:c r="G4" s="8"/>
+      <x:c r="H4" s="8"/>
+      <x:c r="I4" s="8"/>
+      <x:c r="J4" s="8"/>
+      <x:c r="K4" s="8"/>
+      <x:c r="L4" s="8"/>
+      <x:c r="M4" s="8"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
@@ -404,16 +406,16 @@
       <x:c r="C5" s="8" t="str">
         <x:v>Value to include in SMS</x:v>
       </x:c>
-      <x:c r="D5" s="8" t="str"/>
-      <x:c r="E5" s="8" t="str"/>
-      <x:c r="F5" s="8" t="str"/>
-      <x:c r="G5" s="8" t="str"/>
-      <x:c r="H5" s="8" t="str"/>
-      <x:c r="I5" s="8" t="str"/>
-      <x:c r="J5" s="8" t="str"/>
-      <x:c r="K5" s="8" t="str"/>
-      <x:c r="L5" s="8" t="str"/>
-      <x:c r="M5" s="8" t="str"/>
+      <x:c r="D5" s="8"/>
+      <x:c r="E5" s="8"/>
+      <x:c r="F5" s="8"/>
+      <x:c r="G5" s="8"/>
+      <x:c r="H5" s="8"/>
+      <x:c r="I5" s="8"/>
+      <x:c r="J5" s="8"/>
+      <x:c r="K5" s="8"/>
+      <x:c r="L5" s="8"/>
+      <x:c r="M5" s="8"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
@@ -422,19 +424,19 @@
       <x:c r="B6" s="8" t="str">
         <x:v>sms_message_calc</x:v>
       </x:c>
-      <x:c r="C6" s="8" t="str"/>
-      <x:c r="D6" s="8" t="str"/>
-      <x:c r="E6" s="8" t="str"/>
-      <x:c r="F6" s="8" t="str"/>
-      <x:c r="G6" s="8" t="str"/>
-      <x:c r="H6" s="8" t="str"/>
-      <x:c r="I6" s="8" t="str"/>
+      <x:c r="C6" s="8"/>
+      <x:c r="D6" s="8"/>
+      <x:c r="E6" s="8"/>
+      <x:c r="F6" s="8"/>
+      <x:c r="G6" s="8"/>
+      <x:c r="H6" s="8"/>
+      <x:c r="I6" s="8"/>
       <x:c r="J6" s="8" t="str">
         <x:v>concat('Your study code is ', ${field_value}, '.')</x:v>
       </x:c>
-      <x:c r="K6" s="8" t="str"/>
-      <x:c r="L6" s="8" t="str"/>
-      <x:c r="M6" s="8" t="str"/>
+      <x:c r="K6" s="8"/>
+      <x:c r="L6" s="8"/>
+      <x:c r="M6" s="8"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8" t="str">
@@ -452,16 +454,16 @@
       <x:c r="E7" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F7" s="8" t="str"/>
-      <x:c r="G7" s="8" t="str"/>
-      <x:c r="H7" s="8" t="str"/>
-      <x:c r="I7" s="8" t="str"/>
-      <x:c r="J7" s="8" t="str"/>
-      <x:c r="K7" s="8" t="str"/>
+      <x:c r="F7" s="8"/>
+      <x:c r="G7" s="8"/>
+      <x:c r="H7" s="8"/>
+      <x:c r="I7" s="8"/>
+      <x:c r="J7" s="8"/>
+      <x:c r="K7" s="8"/>
       <x:c r="L7" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M7" s="8" t="str"/>
+      <x:c r="M7" s="8"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8" t="str">
@@ -479,16 +481,16 @@
       <x:c r="E8" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F8" s="8" t="str"/>
-      <x:c r="G8" s="8" t="str"/>
-      <x:c r="H8" s="8" t="str"/>
-      <x:c r="I8" s="8" t="str"/>
-      <x:c r="J8" s="8" t="str"/>
-      <x:c r="K8" s="8" t="str"/>
+      <x:c r="F8" s="8"/>
+      <x:c r="G8" s="8"/>
+      <x:c r="H8" s="8"/>
+      <x:c r="I8" s="8"/>
+      <x:c r="J8" s="8"/>
+      <x:c r="K8" s="8"/>
       <x:c r="L8" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M8" s="8" t="str"/>
+      <x:c r="M8" s="8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8" t="str">
@@ -506,16 +508,16 @@
       <x:c r="E9" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F9" s="8" t="str"/>
-      <x:c r="G9" s="8" t="str"/>
-      <x:c r="H9" s="8" t="str"/>
-      <x:c r="I9" s="8" t="str"/>
-      <x:c r="J9" s="8" t="str"/>
-      <x:c r="K9" s="8" t="str"/>
+      <x:c r="F9" s="8"/>
+      <x:c r="G9" s="8"/>
+      <x:c r="H9" s="8"/>
+      <x:c r="I9" s="8"/>
+      <x:c r="J9" s="8"/>
+      <x:c r="K9" s="8"/>
       <x:c r="L9" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M9" s="8" t="str"/>
+      <x:c r="M9" s="8"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
@@ -533,16 +535,16 @@
       <x:c r="E10" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F10" s="8" t="str"/>
-      <x:c r="G10" s="8" t="str"/>
-      <x:c r="H10" s="8" t="str"/>
-      <x:c r="I10" s="8" t="str"/>
-      <x:c r="J10" s="8" t="str"/>
-      <x:c r="K10" s="8" t="str"/>
+      <x:c r="F10" s="8"/>
+      <x:c r="G10" s="8"/>
+      <x:c r="H10" s="8"/>
+      <x:c r="I10" s="8"/>
+      <x:c r="J10" s="8"/>
+      <x:c r="K10" s="8"/>
       <x:c r="L10" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M10" s="8" t="str"/>
+      <x:c r="M10" s="8"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
@@ -560,16 +562,16 @@
       <x:c r="E11" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F11" s="8" t="str"/>
-      <x:c r="G11" s="8" t="str"/>
-      <x:c r="H11" s="8" t="str"/>
-      <x:c r="I11" s="8" t="str"/>
-      <x:c r="J11" s="8" t="str"/>
-      <x:c r="K11" s="8" t="str"/>
+      <x:c r="F11" s="8"/>
+      <x:c r="G11" s="8"/>
+      <x:c r="H11" s="8"/>
+      <x:c r="I11" s="8"/>
+      <x:c r="J11" s="8"/>
+      <x:c r="K11" s="8"/>
       <x:c r="L11" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M11" s="8" t="str"/>
+      <x:c r="M11" s="8"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
@@ -587,16 +589,16 @@
       <x:c r="E12" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F12" s="8" t="str"/>
-      <x:c r="G12" s="8" t="str"/>
-      <x:c r="H12" s="8" t="str"/>
-      <x:c r="I12" s="8" t="str"/>
-      <x:c r="J12" s="8" t="str"/>
-      <x:c r="K12" s="8" t="str"/>
+      <x:c r="F12" s="8"/>
+      <x:c r="G12" s="8"/>
+      <x:c r="H12" s="8"/>
+      <x:c r="I12" s="8"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="8"/>
       <x:c r="L12" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M12" s="8" t="str"/>
+      <x:c r="M12" s="8"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
@@ -614,16 +616,16 @@
       <x:c r="E13" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F13" s="8" t="str"/>
-      <x:c r="G13" s="8" t="str"/>
-      <x:c r="H13" s="8" t="str"/>
-      <x:c r="I13" s="8" t="str"/>
-      <x:c r="J13" s="8" t="str"/>
-      <x:c r="K13" s="8" t="str"/>
+      <x:c r="F13" s="8"/>
+      <x:c r="G13" s="8"/>
+      <x:c r="H13" s="8"/>
+      <x:c r="I13" s="8"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="8"/>
       <x:c r="L13" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M13" s="8" t="str"/>
+      <x:c r="M13" s="8"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
@@ -641,16 +643,16 @@
       <x:c r="E14" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F14" s="8" t="str"/>
-      <x:c r="G14" s="8" t="str"/>
-      <x:c r="H14" s="8" t="str"/>
-      <x:c r="I14" s="8" t="str"/>
-      <x:c r="J14" s="8" t="str"/>
-      <x:c r="K14" s="8" t="str"/>
+      <x:c r="F14" s="8"/>
+      <x:c r="G14" s="8"/>
+      <x:c r="H14" s="8"/>
+      <x:c r="I14" s="8"/>
+      <x:c r="J14" s="8"/>
+      <x:c r="K14" s="8"/>
       <x:c r="L14" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M14" s="8" t="str"/>
+      <x:c r="M14" s="8"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
@@ -668,16 +670,16 @@
       <x:c r="E15" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F15" s="8" t="str"/>
-      <x:c r="G15" s="8" t="str"/>
-      <x:c r="H15" s="8" t="str"/>
-      <x:c r="I15" s="8" t="str"/>
-      <x:c r="J15" s="8" t="str"/>
-      <x:c r="K15" s="8" t="str"/>
+      <x:c r="F15" s="8"/>
+      <x:c r="G15" s="8"/>
+      <x:c r="H15" s="8"/>
+      <x:c r="I15" s="8"/>
+      <x:c r="J15" s="8"/>
+      <x:c r="K15" s="8"/>
       <x:c r="L15" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M15" s="8" t="str"/>
+      <x:c r="M15" s="8"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
@@ -695,56 +697,131 @@
       <x:c r="E16" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F16" s="8" t="str"/>
-      <x:c r="G16" s="8" t="str"/>
-      <x:c r="H16" s="8" t="str"/>
-      <x:c r="I16" s="8" t="str"/>
-      <x:c r="J16" s="8" t="str"/>
-      <x:c r="K16" s="8" t="str"/>
+      <x:c r="F16" s="8"/>
+      <x:c r="G16" s="8"/>
+      <x:c r="H16" s="8"/>
+      <x:c r="I16" s="8"/>
+      <x:c r="J16" s="8"/>
+      <x:c r="K16" s="8"/>
       <x:c r="L16" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M16" s="8" t="str"/>
+      <x:c r="M16" s="8"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
         <x:v>end_group</x:v>
       </x:c>
-      <x:c r="B17" s="8" t="str"/>
-      <x:c r="C17" s="8" t="str"/>
-      <x:c r="D17" s="8" t="str"/>
-      <x:c r="E17" s="8" t="str"/>
-      <x:c r="F17" s="8" t="str"/>
-      <x:c r="G17" s="8" t="str"/>
-      <x:c r="H17" s="8" t="str"/>
-      <x:c r="I17" s="8" t="str"/>
-      <x:c r="J17" s="8" t="str"/>
-      <x:c r="K17" s="8" t="str"/>
-      <x:c r="L17" s="8" t="str"/>
-      <x:c r="M17" s="8" t="str"/>
+      <x:c r="B17" s="8"/>
+      <x:c r="C17" s="8"/>
+      <x:c r="D17" s="8"/>
+      <x:c r="E17" s="8"/>
+      <x:c r="F17" s="8"/>
+      <x:c r="G17" s="8"/>
+      <x:c r="H17" s="8"/>
+      <x:c r="I17" s="8"/>
+      <x:c r="J17" s="8"/>
+      <x:c r="K17" s="8"/>
+      <x:c r="L17" s="8"/>
+      <x:c r="M17" s="8"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>sms_recipients_json</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>SMS recipients JSON</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E18" s="8"/>
+      <x:c r="F18" s="8"/>
+      <x:c r="G18" s="8"/>
+      <x:c r="H18" s="8"/>
+      <x:c r="I18" s="8"/>
+      <x:c r="J18" s="8"/>
+      <x:c r="K18" s="8"/>
+      <x:c r="L18" s="8" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M18" s="8"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>sms_recipient_count</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>SMS recipient count</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
+      <x:c r="K19"/>
+      <x:c r="L19" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>sms_recipient_results_json</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>SMS recipient results JSON</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
+      <x:c r="K20"/>
+      <x:c r="L20" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
         <x:v>note</x:v>
       </x:c>
-      <x:c r="B18" s="8" t="str">
+      <x:c r="B21" t="str">
         <x:v>return_summary</x:v>
       </x:c>
-      <x:c r="C18" s="8" t="str">
+      <x:c r="C21" t="str">
         <x:v>MethodMesh return captured. Status: ${methodmesh_status}</x:v>
       </x:c>
-      <x:c r="D18" s="8" t="str">
+      <x:c r="D21" t="str">
         <x:v>Only fields relevant to this capability are stored, plus the shared FULL envelope.</x:v>
       </x:c>
-      <x:c r="E18" s="8" t="str"/>
-      <x:c r="F18" s="8" t="str"/>
-      <x:c r="G18" s="8" t="str"/>
-      <x:c r="H18" s="8" t="str"/>
-      <x:c r="I18" s="8" t="str"/>
-      <x:c r="J18" s="8" t="str"/>
-      <x:c r="K18" s="8" t="str"/>
-      <x:c r="L18" s="8" t="str"/>
-      <x:c r="M18" s="8" t="str"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
+      <x:c r="K21"/>
+      <x:c r="L21"/>
+      <x:c r="M21"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -804,7 +881,7 @@
         <x:v>sms_sms_send</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>2026090701</x:v>
+        <x:v>2026101602</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>